<commit_message>
css maybe changed? it wanted to be saved
</commit_message>
<xml_diff>
--- a/content/shows/2026/At_This_Moment_Invneotry_Wall Labels.xlsx
+++ b/content/shows/2026/At_This_Moment_Invneotry_Wall Labels.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Exhibition\2026 Shows\At This Moment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\atthismoment\content\shows\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09EF2F51-BAFB-489F-BD79-92AD7155C0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{627D0C7A-AF8E-434F-AF86-C7A8FD6A414E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -889,7 +889,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -966,10 +966,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1310,21 +1310,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I47"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.796875" style="3"/>
-    <col min="2" max="2" width="14.69921875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="29.69921875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="22.09765625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.796875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="3"/>
+    <col min="2" max="2" width="14.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="22.08203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" style="3" customWidth="1"/>
     <col min="6" max="6" width="23.5" style="3" customWidth="1"/>
-    <col min="7" max="7" width="47.09765625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="39.296875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="8.796875" style="5"/>
-    <col min="10" max="16384" width="8.796875" style="3"/>
+    <col min="7" max="7" width="47.08203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="39.33203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" style="5"/>
+    <col min="10" max="16384" width="8.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>107</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="62" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>49</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="62" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>49</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>203</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>203</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>270</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>212</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>179</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>168</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>168</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="62" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>123</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>89</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>237</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>130</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="31" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>130</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="78" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>244</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>162</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="62" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>138</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="78" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>138</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>138</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>66</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>59</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>97</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>97</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="156" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>10</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="78" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="62" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>114</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>39</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>39</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>187</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>131</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>155</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="93" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>250</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>250</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>75</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>75</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>75</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="78" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>226</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>169</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>169</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="124" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>195</v>
       </c>
@@ -2427,7 +2427,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>195</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="78" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
         <v>64</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>28</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" ht="62" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>28</v>
       </c>

</xml_diff>